<commit_message>
Remove Etretat from day 5, keep Bayeux+Omaha in order, add D-Day Memorial note; update HTML, Excel and KML.
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v4/itinerary.xlsx
+++ b/v4/itinerary.xlsx
@@ -831,32 +831,32 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Bayeux + Omaha + Etretat</t>
+          <t>Bayeux + Omaha Beach</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>~260 km</t>
+          <t>~250 km</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Partenza ore 7:00. A13 -&gt; Caen -&gt; Bayeux (~2h30): Arazzo XI sec. (70m, 1h), cattedrale. Omaha Beach + Cimitero Americano Colleville-sur-Mer. Pointe du Hoc: trincee e crateri intatti. Pranzo a Port-en-Bessin.</t>
+          <t>Partenza ore 7:00. A13 -&gt; Caen -&gt; Bayeux (~2h30): Arazzo XI sec. (70m, 1h), cattedrale. Pranzo a Port-en-Bessin (porto peschereccio, ottimo pesce fresco).</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Etretat (15:00): scogliere bianche piu famose d'Europa, passeggiata sulle falaise (1h, facile). Tramonto spettacolare da lassu.</t>
+          <t>Omaha Beach + Memoriale Nazionale D-Day (National D-Day Memorial): museo all'aperto, installazioni emozionanti, accessibile per i bambini. Cimitero Americano di Colleville-sur-Mer. Pointe du Hoc: trincee e crateri intatti.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Camping Municipal d'Etretat ***</t>
+          <t>Camping Port'land - Port-en-Bessin ***** (sul porto, piscina coperta)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Camping Port'land - Port-en-Bessin *****</t>
+          <t>Camping de Bayeux ****</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Replace Aosta with Courmayeur as first night stop, fix day 1 route description, update HTML/Excel/KML.
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v4/itinerary.xlsx
+++ b/v4/itinerary.xlsx
@@ -631,22 +631,22 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Milano -&gt; Aosta</t>
+          <t>Milano -&gt; Courmayeur</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>~110 km</t>
+          <t>~140 km</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Ritiro camper ore 15:00. Partenza ore 19:00 da Milano. A4 Torino -&gt; Traforo del Frejus (~60EUR/camper) -&gt; Aosta. Solo 110 km: familiarizzazione con il camper senza stress.</t>
+          <t>Ritiro camper ore 15:00 - verificare tutto sul posto. Partenza ore 19:00 da Milano. A4 -&gt; Torino -&gt; A5 -&gt; Aosta -&gt; Courmayeur. ~140 km: guida tranquilla per familiarizzare col camper.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Arrivo Aosta/Courmayeur ~21:00. Prima sistemazione, cena di gruppo. I bambini esplorano il camper!</t>
+          <t>Arrivo Courmayeur ~21:30. Prima sistemazione camper, cena di gruppo. I bambini esplorano il camper! Notte rilassata - domani Traforo Monte Bianco.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Camping Milleluci - Aosta ****</t>
+          <t>Camping Gran Paradiso - Villeneuve AO ****</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Aosta -&gt; Versailles</t>
+          <t>Courmayeur -&gt; Versailles</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">

</xml_diff>